<commit_message>
Add employee schedule web app with form, approval workflow, and visual timeline
- Flask app (app.py): employees submit shift times + lunch via tokenised email
  link; manager reviews, approves or requests changes; employees can accept
  changes with one click or reopen the form to modify
- 6 HTML templates: employee form, manager dashboard (up to 15 employees),
  review/edit page, login, submitted, error
- Excel export: Schedule Summary tab + Visual Timeline tab — one row per
  employee per weekday (Mon–Fri), 30-min columns 8 AM–9 PM, on-shift cells
  blue, lunch yellow, off-shift empty; scroll vertically to compare employees
- config.json: employee list, SMTP settings, manager password
- generate_schedule.py updated to include same visual timeline as third tab

https://claude.ai/code/session_01CZvMQ2DgKz2CDzsDjTf1FF
</commit_message>
<xml_diff>
--- a/employee_weekly_schedule.xlsx
+++ b/employee_weekly_schedule.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Weekly Schedule" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Blank Template" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Visual Timeline" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Weekly Schedule'!$1:$5</definedName>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -74,8 +75,39 @@
       <color rgb="00000000"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="7"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001F4E79"/>
+      <sz val="7"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="19">
     <fill>
       <patternFill/>
     </fill>
@@ -142,8 +174,33 @@
         <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBF3FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F6FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F0F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FAFAFA"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="12">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -293,11 +350,71 @@
         <color rgb="001F4E79"/>
       </bottom>
     </border>
+    <border>
+      <left style="hair">
+        <color rgb="00DDDDDD"/>
+      </left>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <bottom style="hair">
+        <color rgb="00E0E0E0"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="hair">
+        <color rgb="00D8D8D8"/>
+      </left>
+      <bottom style="hair">
+        <color rgb="00E0E0E0"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <bottom style="medium">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="hair">
+        <color rgb="00D8D8D8"/>
+      </left>
+      <bottom style="medium">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="001F4E79"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="medium">
+        <color rgb="001F4E79"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="001F4E79"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -437,6 +554,57 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="17" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="14" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="18" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="18" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="18" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1762,4 +1930,1602 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:AB52"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="2.6" customWidth="1" min="3" max="3"/>
+    <col width="2.6" customWidth="1" min="4" max="4"/>
+    <col width="2.6" customWidth="1" min="5" max="5"/>
+    <col width="2.6" customWidth="1" min="6" max="6"/>
+    <col width="2.6" customWidth="1" min="7" max="7"/>
+    <col width="2.6" customWidth="1" min="8" max="8"/>
+    <col width="2.6" customWidth="1" min="9" max="9"/>
+    <col width="2.6" customWidth="1" min="10" max="10"/>
+    <col width="2.6" customWidth="1" min="11" max="11"/>
+    <col width="2.6" customWidth="1" min="12" max="12"/>
+    <col width="2.6" customWidth="1" min="13" max="13"/>
+    <col width="2.6" customWidth="1" min="14" max="14"/>
+    <col width="2.6" customWidth="1" min="15" max="15"/>
+    <col width="2.6" customWidth="1" min="16" max="16"/>
+    <col width="2.6" customWidth="1" min="17" max="17"/>
+    <col width="2.6" customWidth="1" min="18" max="18"/>
+    <col width="2.6" customWidth="1" min="19" max="19"/>
+    <col width="2.6" customWidth="1" min="20" max="20"/>
+    <col width="2.6" customWidth="1" min="21" max="21"/>
+    <col width="2.6" customWidth="1" min="22" max="22"/>
+    <col width="2.6" customWidth="1" min="23" max="23"/>
+    <col width="2.6" customWidth="1" min="24" max="24"/>
+    <col width="2.6" customWidth="1" min="25" max="25"/>
+    <col width="2.6" customWidth="1" min="26" max="26"/>
+    <col width="2.6" customWidth="1" min="27" max="27"/>
+    <col width="2.6" customWidth="1" min="28" max="28"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="49" t="inlineStr">
+        <is>
+          <t>Staff Coverage Timeline  —  Week of June 15, 2026  (Mon–Fri  |  8 AM – 9 PM  |  30-min slots)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="50" t="inlineStr">
+        <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="B2" s="50" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="C2" s="51" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D2" s="52" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="E2" s="51" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="F2" s="52" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="G2" s="51" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="H2" s="52" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="I2" s="51" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="J2" s="52" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="K2" s="51" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="L2" s="52" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="M2" s="51" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="N2" s="52" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="O2" s="51" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="P2" s="52" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="Q2" s="51" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="R2" s="52" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="S2" s="51" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="T2" s="52" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="U2" s="51" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="V2" s="52" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="W2" s="51" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="X2" s="52" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="Y2" s="51" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="Z2" s="52" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="AA2" s="51" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="AB2" s="52" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="53" t="inlineStr">
+        <is>
+          <t>Alice Johnson</t>
+        </is>
+      </c>
+      <c r="B3" s="54" t="inlineStr">
+        <is>
+          <t>Mon  06/15</t>
+        </is>
+      </c>
+      <c r="C3" s="55" t="n"/>
+      <c r="D3" s="55" t="n"/>
+      <c r="E3" s="55" t="n"/>
+      <c r="F3" s="55" t="n"/>
+      <c r="G3" s="55" t="n"/>
+      <c r="H3" s="55" t="n"/>
+      <c r="I3" s="56" t="n"/>
+      <c r="J3" s="55" t="n"/>
+      <c r="K3" s="55" t="n"/>
+      <c r="L3" s="55" t="n"/>
+      <c r="M3" s="55" t="n"/>
+      <c r="N3" s="55" t="n"/>
+      <c r="O3" s="57" t="n"/>
+      <c r="P3" s="57" t="n"/>
+      <c r="Q3" s="57" t="n"/>
+      <c r="R3" s="57" t="n"/>
+      <c r="S3" s="57" t="n"/>
+      <c r="T3" s="57" t="n"/>
+      <c r="U3" s="57" t="n"/>
+      <c r="V3" s="57" t="n"/>
+      <c r="W3" s="57" t="n"/>
+      <c r="X3" s="57" t="n"/>
+      <c r="Y3" s="57" t="n"/>
+      <c r="Z3" s="57" t="n"/>
+      <c r="AA3" s="57" t="n"/>
+      <c r="AB3" s="57" t="n"/>
+    </row>
+    <row r="4" ht="16" customHeight="1">
+      <c r="B4" s="58" t="inlineStr">
+        <is>
+          <t>Tue  06/16</t>
+        </is>
+      </c>
+      <c r="C4" s="55" t="n"/>
+      <c r="D4" s="55" t="n"/>
+      <c r="E4" s="55" t="n"/>
+      <c r="F4" s="55" t="n"/>
+      <c r="G4" s="55" t="n"/>
+      <c r="H4" s="55" t="n"/>
+      <c r="I4" s="56" t="n"/>
+      <c r="J4" s="55" t="n"/>
+      <c r="K4" s="55" t="n"/>
+      <c r="L4" s="55" t="n"/>
+      <c r="M4" s="55" t="n"/>
+      <c r="N4" s="55" t="n"/>
+      <c r="O4" s="57" t="n"/>
+      <c r="P4" s="57" t="n"/>
+      <c r="Q4" s="57" t="n"/>
+      <c r="R4" s="57" t="n"/>
+      <c r="S4" s="57" t="n"/>
+      <c r="T4" s="57" t="n"/>
+      <c r="U4" s="57" t="n"/>
+      <c r="V4" s="57" t="n"/>
+      <c r="W4" s="57" t="n"/>
+      <c r="X4" s="57" t="n"/>
+      <c r="Y4" s="57" t="n"/>
+      <c r="Z4" s="57" t="n"/>
+      <c r="AA4" s="57" t="n"/>
+      <c r="AB4" s="57" t="n"/>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="B5" s="58" t="inlineStr">
+        <is>
+          <t>Wed  06/17</t>
+        </is>
+      </c>
+      <c r="C5" s="55" t="n"/>
+      <c r="D5" s="55" t="n"/>
+      <c r="E5" s="55" t="n"/>
+      <c r="F5" s="55" t="n"/>
+      <c r="G5" s="55" t="n"/>
+      <c r="H5" s="55" t="n"/>
+      <c r="I5" s="56" t="n"/>
+      <c r="J5" s="55" t="n"/>
+      <c r="K5" s="55" t="n"/>
+      <c r="L5" s="55" t="n"/>
+      <c r="M5" s="55" t="n"/>
+      <c r="N5" s="55" t="n"/>
+      <c r="O5" s="57" t="n"/>
+      <c r="P5" s="57" t="n"/>
+      <c r="Q5" s="57" t="n"/>
+      <c r="R5" s="57" t="n"/>
+      <c r="S5" s="57" t="n"/>
+      <c r="T5" s="57" t="n"/>
+      <c r="U5" s="57" t="n"/>
+      <c r="V5" s="57" t="n"/>
+      <c r="W5" s="57" t="n"/>
+      <c r="X5" s="57" t="n"/>
+      <c r="Y5" s="57" t="n"/>
+      <c r="Z5" s="57" t="n"/>
+      <c r="AA5" s="57" t="n"/>
+      <c r="AB5" s="57" t="n"/>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="B6" s="58" t="inlineStr">
+        <is>
+          <t>Thu  06/18</t>
+        </is>
+      </c>
+      <c r="C6" s="55" t="n"/>
+      <c r="D6" s="55" t="n"/>
+      <c r="E6" s="55" t="n"/>
+      <c r="F6" s="55" t="n"/>
+      <c r="G6" s="55" t="n"/>
+      <c r="H6" s="55" t="n"/>
+      <c r="I6" s="56" t="n"/>
+      <c r="J6" s="55" t="n"/>
+      <c r="K6" s="55" t="n"/>
+      <c r="L6" s="55" t="n"/>
+      <c r="M6" s="55" t="n"/>
+      <c r="N6" s="55" t="n"/>
+      <c r="O6" s="57" t="n"/>
+      <c r="P6" s="57" t="n"/>
+      <c r="Q6" s="57" t="n"/>
+      <c r="R6" s="57" t="n"/>
+      <c r="S6" s="57" t="n"/>
+      <c r="T6" s="57" t="n"/>
+      <c r="U6" s="57" t="n"/>
+      <c r="V6" s="57" t="n"/>
+      <c r="W6" s="57" t="n"/>
+      <c r="X6" s="57" t="n"/>
+      <c r="Y6" s="57" t="n"/>
+      <c r="Z6" s="57" t="n"/>
+      <c r="AA6" s="57" t="n"/>
+      <c r="AB6" s="57" t="n"/>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="B7" s="59" t="inlineStr">
+        <is>
+          <t>Fri  06/19</t>
+        </is>
+      </c>
+      <c r="C7" s="60" t="n"/>
+      <c r="D7" s="60" t="n"/>
+      <c r="E7" s="60" t="n"/>
+      <c r="F7" s="60" t="n"/>
+      <c r="G7" s="60" t="n"/>
+      <c r="H7" s="60" t="n"/>
+      <c r="I7" s="61" t="n"/>
+      <c r="J7" s="60" t="n"/>
+      <c r="K7" s="60" t="n"/>
+      <c r="L7" s="60" t="n"/>
+      <c r="M7" s="60" t="n"/>
+      <c r="N7" s="60" t="n"/>
+      <c r="O7" s="62" t="n"/>
+      <c r="P7" s="62" t="n"/>
+      <c r="Q7" s="62" t="n"/>
+      <c r="R7" s="62" t="n"/>
+      <c r="S7" s="62" t="n"/>
+      <c r="T7" s="62" t="n"/>
+      <c r="U7" s="62" t="n"/>
+      <c r="V7" s="62" t="n"/>
+      <c r="W7" s="62" t="n"/>
+      <c r="X7" s="62" t="n"/>
+      <c r="Y7" s="62" t="n"/>
+      <c r="Z7" s="62" t="n"/>
+      <c r="AA7" s="62" t="n"/>
+      <c r="AB7" s="62" t="n"/>
+    </row>
+    <row r="8" ht="4" customHeight="1"/>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="63" t="inlineStr">
+        <is>
+          <t>Bob Martinez</t>
+        </is>
+      </c>
+      <c r="B9" s="64" t="inlineStr">
+        <is>
+          <t>Mon  06/15</t>
+        </is>
+      </c>
+      <c r="C9" s="65" t="n"/>
+      <c r="D9" s="65" t="n"/>
+      <c r="E9" s="65" t="n"/>
+      <c r="F9" s="65" t="n"/>
+      <c r="G9" s="65" t="n"/>
+      <c r="H9" s="65" t="n"/>
+      <c r="I9" s="65" t="n"/>
+      <c r="J9" s="65" t="n"/>
+      <c r="K9" s="65" t="n"/>
+      <c r="L9" s="65" t="n"/>
+      <c r="M9" s="65" t="n"/>
+      <c r="N9" s="65" t="n"/>
+      <c r="O9" s="55" t="n"/>
+      <c r="P9" s="55" t="n"/>
+      <c r="Q9" s="55" t="n"/>
+      <c r="R9" s="55" t="n"/>
+      <c r="S9" s="55" t="n"/>
+      <c r="T9" s="55" t="n"/>
+      <c r="U9" s="55" t="n"/>
+      <c r="V9" s="56" t="n"/>
+      <c r="W9" s="55" t="n"/>
+      <c r="X9" s="55" t="n"/>
+      <c r="Y9" s="55" t="n"/>
+      <c r="Z9" s="55" t="n"/>
+      <c r="AA9" s="55" t="n"/>
+      <c r="AB9" s="55" t="n"/>
+    </row>
+    <row r="10" ht="16" customHeight="1">
+      <c r="B10" s="66" t="inlineStr">
+        <is>
+          <t>Tue  06/16</t>
+        </is>
+      </c>
+      <c r="C10" s="65" t="n"/>
+      <c r="D10" s="65" t="n"/>
+      <c r="E10" s="65" t="n"/>
+      <c r="F10" s="65" t="n"/>
+      <c r="G10" s="65" t="n"/>
+      <c r="H10" s="65" t="n"/>
+      <c r="I10" s="65" t="n"/>
+      <c r="J10" s="65" t="n"/>
+      <c r="K10" s="65" t="n"/>
+      <c r="L10" s="65" t="n"/>
+      <c r="M10" s="65" t="n"/>
+      <c r="N10" s="65" t="n"/>
+      <c r="O10" s="55" t="n"/>
+      <c r="P10" s="55" t="n"/>
+      <c r="Q10" s="55" t="n"/>
+      <c r="R10" s="55" t="n"/>
+      <c r="S10" s="55" t="n"/>
+      <c r="T10" s="55" t="n"/>
+      <c r="U10" s="55" t="n"/>
+      <c r="V10" s="56" t="n"/>
+      <c r="W10" s="55" t="n"/>
+      <c r="X10" s="55" t="n"/>
+      <c r="Y10" s="55" t="n"/>
+      <c r="Z10" s="55" t="n"/>
+      <c r="AA10" s="55" t="n"/>
+      <c r="AB10" s="55" t="n"/>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="B11" s="66" t="inlineStr">
+        <is>
+          <t>Wed  06/17</t>
+        </is>
+      </c>
+      <c r="C11" s="65" t="n"/>
+      <c r="D11" s="65" t="n"/>
+      <c r="E11" s="65" t="n"/>
+      <c r="F11" s="65" t="n"/>
+      <c r="G11" s="65" t="n"/>
+      <c r="H11" s="65" t="n"/>
+      <c r="I11" s="65" t="n"/>
+      <c r="J11" s="65" t="n"/>
+      <c r="K11" s="65" t="n"/>
+      <c r="L11" s="65" t="n"/>
+      <c r="M11" s="65" t="n"/>
+      <c r="N11" s="65" t="n"/>
+      <c r="O11" s="65" t="n"/>
+      <c r="P11" s="65" t="n"/>
+      <c r="Q11" s="65" t="n"/>
+      <c r="R11" s="65" t="n"/>
+      <c r="S11" s="65" t="n"/>
+      <c r="T11" s="65" t="n"/>
+      <c r="U11" s="65" t="n"/>
+      <c r="V11" s="65" t="n"/>
+      <c r="W11" s="65" t="n"/>
+      <c r="X11" s="65" t="n"/>
+      <c r="Y11" s="65" t="n"/>
+      <c r="Z11" s="65" t="n"/>
+      <c r="AA11" s="65" t="n"/>
+      <c r="AB11" s="65" t="n"/>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="B12" s="66" t="inlineStr">
+        <is>
+          <t>Thu  06/18</t>
+        </is>
+      </c>
+      <c r="C12" s="65" t="n"/>
+      <c r="D12" s="65" t="n"/>
+      <c r="E12" s="65" t="n"/>
+      <c r="F12" s="65" t="n"/>
+      <c r="G12" s="65" t="n"/>
+      <c r="H12" s="65" t="n"/>
+      <c r="I12" s="65" t="n"/>
+      <c r="J12" s="65" t="n"/>
+      <c r="K12" s="65" t="n"/>
+      <c r="L12" s="65" t="n"/>
+      <c r="M12" s="65" t="n"/>
+      <c r="N12" s="65" t="n"/>
+      <c r="O12" s="55" t="n"/>
+      <c r="P12" s="55" t="n"/>
+      <c r="Q12" s="55" t="n"/>
+      <c r="R12" s="55" t="n"/>
+      <c r="S12" s="55" t="n"/>
+      <c r="T12" s="55" t="n"/>
+      <c r="U12" s="55" t="n"/>
+      <c r="V12" s="56" t="n"/>
+      <c r="W12" s="55" t="n"/>
+      <c r="X12" s="55" t="n"/>
+      <c r="Y12" s="55" t="n"/>
+      <c r="Z12" s="55" t="n"/>
+      <c r="AA12" s="55" t="n"/>
+      <c r="AB12" s="55" t="n"/>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="B13" s="67" t="inlineStr">
+        <is>
+          <t>Fri  06/19</t>
+        </is>
+      </c>
+      <c r="C13" s="68" t="n"/>
+      <c r="D13" s="68" t="n"/>
+      <c r="E13" s="68" t="n"/>
+      <c r="F13" s="68" t="n"/>
+      <c r="G13" s="68" t="n"/>
+      <c r="H13" s="68" t="n"/>
+      <c r="I13" s="68" t="n"/>
+      <c r="J13" s="68" t="n"/>
+      <c r="K13" s="68" t="n"/>
+      <c r="L13" s="68" t="n"/>
+      <c r="M13" s="68" t="n"/>
+      <c r="N13" s="68" t="n"/>
+      <c r="O13" s="60" t="n"/>
+      <c r="P13" s="60" t="n"/>
+      <c r="Q13" s="60" t="n"/>
+      <c r="R13" s="60" t="n"/>
+      <c r="S13" s="60" t="n"/>
+      <c r="T13" s="60" t="n"/>
+      <c r="U13" s="60" t="n"/>
+      <c r="V13" s="61" t="n"/>
+      <c r="W13" s="60" t="n"/>
+      <c r="X13" s="60" t="n"/>
+      <c r="Y13" s="60" t="n"/>
+      <c r="Z13" s="60" t="n"/>
+      <c r="AA13" s="60" t="n"/>
+      <c r="AB13" s="60" t="n"/>
+    </row>
+    <row r="14" ht="4" customHeight="1"/>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="53" t="inlineStr">
+        <is>
+          <t>Carol Smith</t>
+        </is>
+      </c>
+      <c r="B15" s="54" t="inlineStr">
+        <is>
+          <t>Mon  06/15</t>
+        </is>
+      </c>
+      <c r="C15" s="55" t="n"/>
+      <c r="D15" s="55" t="n"/>
+      <c r="E15" s="55" t="n"/>
+      <c r="F15" s="55" t="n"/>
+      <c r="G15" s="55" t="n"/>
+      <c r="H15" s="55" t="n"/>
+      <c r="I15" s="55" t="n"/>
+      <c r="J15" s="55" t="n"/>
+      <c r="K15" s="56" t="n"/>
+      <c r="L15" s="55" t="n"/>
+      <c r="M15" s="55" t="n"/>
+      <c r="N15" s="55" t="n"/>
+      <c r="O15" s="55" t="n"/>
+      <c r="P15" s="55" t="n"/>
+      <c r="Q15" s="55" t="n"/>
+      <c r="R15" s="55" t="n"/>
+      <c r="S15" s="57" t="n"/>
+      <c r="T15" s="57" t="n"/>
+      <c r="U15" s="57" t="n"/>
+      <c r="V15" s="57" t="n"/>
+      <c r="W15" s="57" t="n"/>
+      <c r="X15" s="57" t="n"/>
+      <c r="Y15" s="57" t="n"/>
+      <c r="Z15" s="57" t="n"/>
+      <c r="AA15" s="57" t="n"/>
+      <c r="AB15" s="57" t="n"/>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="B16" s="58" t="inlineStr">
+        <is>
+          <t>Tue  06/16</t>
+        </is>
+      </c>
+      <c r="C16" s="57" t="n"/>
+      <c r="D16" s="57" t="n"/>
+      <c r="E16" s="57" t="n"/>
+      <c r="F16" s="57" t="n"/>
+      <c r="G16" s="57" t="n"/>
+      <c r="H16" s="57" t="n"/>
+      <c r="I16" s="57" t="n"/>
+      <c r="J16" s="57" t="n"/>
+      <c r="K16" s="57" t="n"/>
+      <c r="L16" s="57" t="n"/>
+      <c r="M16" s="57" t="n"/>
+      <c r="N16" s="57" t="n"/>
+      <c r="O16" s="57" t="n"/>
+      <c r="P16" s="57" t="n"/>
+      <c r="Q16" s="57" t="n"/>
+      <c r="R16" s="57" t="n"/>
+      <c r="S16" s="57" t="n"/>
+      <c r="T16" s="57" t="n"/>
+      <c r="U16" s="57" t="n"/>
+      <c r="V16" s="57" t="n"/>
+      <c r="W16" s="57" t="n"/>
+      <c r="X16" s="57" t="n"/>
+      <c r="Y16" s="57" t="n"/>
+      <c r="Z16" s="57" t="n"/>
+      <c r="AA16" s="57" t="n"/>
+      <c r="AB16" s="57" t="n"/>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="B17" s="58" t="inlineStr">
+        <is>
+          <t>Wed  06/17</t>
+        </is>
+      </c>
+      <c r="C17" s="55" t="n"/>
+      <c r="D17" s="55" t="n"/>
+      <c r="E17" s="55" t="n"/>
+      <c r="F17" s="55" t="n"/>
+      <c r="G17" s="55" t="n"/>
+      <c r="H17" s="55" t="n"/>
+      <c r="I17" s="55" t="n"/>
+      <c r="J17" s="55" t="n"/>
+      <c r="K17" s="56" t="n"/>
+      <c r="L17" s="55" t="n"/>
+      <c r="M17" s="55" t="n"/>
+      <c r="N17" s="55" t="n"/>
+      <c r="O17" s="55" t="n"/>
+      <c r="P17" s="55" t="n"/>
+      <c r="Q17" s="55" t="n"/>
+      <c r="R17" s="55" t="n"/>
+      <c r="S17" s="57" t="n"/>
+      <c r="T17" s="57" t="n"/>
+      <c r="U17" s="57" t="n"/>
+      <c r="V17" s="57" t="n"/>
+      <c r="W17" s="57" t="n"/>
+      <c r="X17" s="57" t="n"/>
+      <c r="Y17" s="57" t="n"/>
+      <c r="Z17" s="57" t="n"/>
+      <c r="AA17" s="57" t="n"/>
+      <c r="AB17" s="57" t="n"/>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="B18" s="58" t="inlineStr">
+        <is>
+          <t>Thu  06/18</t>
+        </is>
+      </c>
+      <c r="C18" s="55" t="n"/>
+      <c r="D18" s="55" t="n"/>
+      <c r="E18" s="55" t="n"/>
+      <c r="F18" s="55" t="n"/>
+      <c r="G18" s="55" t="n"/>
+      <c r="H18" s="55" t="n"/>
+      <c r="I18" s="55" t="n"/>
+      <c r="J18" s="55" t="n"/>
+      <c r="K18" s="56" t="n"/>
+      <c r="L18" s="55" t="n"/>
+      <c r="M18" s="55" t="n"/>
+      <c r="N18" s="55" t="n"/>
+      <c r="O18" s="55" t="n"/>
+      <c r="P18" s="55" t="n"/>
+      <c r="Q18" s="55" t="n"/>
+      <c r="R18" s="55" t="n"/>
+      <c r="S18" s="57" t="n"/>
+      <c r="T18" s="57" t="n"/>
+      <c r="U18" s="57" t="n"/>
+      <c r="V18" s="57" t="n"/>
+      <c r="W18" s="57" t="n"/>
+      <c r="X18" s="57" t="n"/>
+      <c r="Y18" s="57" t="n"/>
+      <c r="Z18" s="57" t="n"/>
+      <c r="AA18" s="57" t="n"/>
+      <c r="AB18" s="57" t="n"/>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="B19" s="59" t="inlineStr">
+        <is>
+          <t>Fri  06/19</t>
+        </is>
+      </c>
+      <c r="C19" s="60" t="n"/>
+      <c r="D19" s="60" t="n"/>
+      <c r="E19" s="60" t="n"/>
+      <c r="F19" s="60" t="n"/>
+      <c r="G19" s="60" t="n"/>
+      <c r="H19" s="60" t="n"/>
+      <c r="I19" s="60" t="n"/>
+      <c r="J19" s="60" t="n"/>
+      <c r="K19" s="61" t="n"/>
+      <c r="L19" s="60" t="n"/>
+      <c r="M19" s="60" t="n"/>
+      <c r="N19" s="60" t="n"/>
+      <c r="O19" s="60" t="n"/>
+      <c r="P19" s="60" t="n"/>
+      <c r="Q19" s="60" t="n"/>
+      <c r="R19" s="60" t="n"/>
+      <c r="S19" s="62" t="n"/>
+      <c r="T19" s="62" t="n"/>
+      <c r="U19" s="62" t="n"/>
+      <c r="V19" s="62" t="n"/>
+      <c r="W19" s="62" t="n"/>
+      <c r="X19" s="62" t="n"/>
+      <c r="Y19" s="62" t="n"/>
+      <c r="Z19" s="62" t="n"/>
+      <c r="AA19" s="62" t="n"/>
+      <c r="AB19" s="62" t="n"/>
+    </row>
+    <row r="20" ht="4" customHeight="1"/>
+    <row r="21" ht="16" customHeight="1">
+      <c r="A21" s="63" t="inlineStr">
+        <is>
+          <t>David Lee</t>
+        </is>
+      </c>
+      <c r="B21" s="64" t="inlineStr">
+        <is>
+          <t>Mon  06/15</t>
+        </is>
+      </c>
+      <c r="C21" s="65" t="n"/>
+      <c r="D21" s="65" t="n"/>
+      <c r="E21" s="65" t="n"/>
+      <c r="F21" s="65" t="n"/>
+      <c r="G21" s="65" t="n"/>
+      <c r="H21" s="65" t="n"/>
+      <c r="I21" s="65" t="n"/>
+      <c r="J21" s="65" t="n"/>
+      <c r="K21" s="65" t="n"/>
+      <c r="L21" s="65" t="n"/>
+      <c r="M21" s="65" t="n"/>
+      <c r="N21" s="65" t="n"/>
+      <c r="O21" s="65" t="n"/>
+      <c r="P21" s="65" t="n"/>
+      <c r="Q21" s="65" t="n"/>
+      <c r="R21" s="65" t="n"/>
+      <c r="S21" s="65" t="n"/>
+      <c r="T21" s="65" t="n"/>
+      <c r="U21" s="65" t="n"/>
+      <c r="V21" s="65" t="n"/>
+      <c r="W21" s="65" t="n"/>
+      <c r="X21" s="65" t="n"/>
+      <c r="Y21" s="65" t="n"/>
+      <c r="Z21" s="65" t="n"/>
+      <c r="AA21" s="65" t="n"/>
+      <c r="AB21" s="65" t="n"/>
+    </row>
+    <row r="22" ht="16" customHeight="1">
+      <c r="B22" s="66" t="inlineStr">
+        <is>
+          <t>Tue  06/16</t>
+        </is>
+      </c>
+      <c r="C22" s="65" t="n"/>
+      <c r="D22" s="65" t="n"/>
+      <c r="E22" s="65" t="n"/>
+      <c r="F22" s="65" t="n"/>
+      <c r="G22" s="65" t="n"/>
+      <c r="H22" s="65" t="n"/>
+      <c r="I22" s="65" t="n"/>
+      <c r="J22" s="65" t="n"/>
+      <c r="K22" s="65" t="n"/>
+      <c r="L22" s="65" t="n"/>
+      <c r="M22" s="65" t="n"/>
+      <c r="N22" s="65" t="n"/>
+      <c r="O22" s="65" t="n"/>
+      <c r="P22" s="65" t="n"/>
+      <c r="Q22" s="65" t="n"/>
+      <c r="R22" s="65" t="n"/>
+      <c r="S22" s="65" t="n"/>
+      <c r="T22" s="65" t="n"/>
+      <c r="U22" s="65" t="n"/>
+      <c r="V22" s="65" t="n"/>
+      <c r="W22" s="65" t="n"/>
+      <c r="X22" s="65" t="n"/>
+      <c r="Y22" s="65" t="n"/>
+      <c r="Z22" s="65" t="n"/>
+      <c r="AA22" s="65" t="n"/>
+      <c r="AB22" s="65" t="n"/>
+    </row>
+    <row r="23" ht="16" customHeight="1">
+      <c r="B23" s="66" t="inlineStr">
+        <is>
+          <t>Wed  06/17</t>
+        </is>
+      </c>
+      <c r="C23" s="65" t="n"/>
+      <c r="D23" s="65" t="n"/>
+      <c r="E23" s="65" t="n"/>
+      <c r="F23" s="65" t="n"/>
+      <c r="G23" s="65" t="n"/>
+      <c r="H23" s="65" t="n"/>
+      <c r="I23" s="65" t="n"/>
+      <c r="J23" s="65" t="n"/>
+      <c r="K23" s="65" t="n"/>
+      <c r="L23" s="65" t="n"/>
+      <c r="M23" s="65" t="n"/>
+      <c r="N23" s="65" t="n"/>
+      <c r="O23" s="65" t="n"/>
+      <c r="P23" s="65" t="n"/>
+      <c r="Q23" s="65" t="n"/>
+      <c r="R23" s="65" t="n"/>
+      <c r="S23" s="65" t="n"/>
+      <c r="T23" s="65" t="n"/>
+      <c r="U23" s="65" t="n"/>
+      <c r="V23" s="65" t="n"/>
+      <c r="W23" s="65" t="n"/>
+      <c r="X23" s="65" t="n"/>
+      <c r="Y23" s="65" t="n"/>
+      <c r="Z23" s="65" t="n"/>
+      <c r="AA23" s="65" t="n"/>
+      <c r="AB23" s="65" t="n"/>
+    </row>
+    <row r="24" ht="16" customHeight="1">
+      <c r="B24" s="66" t="inlineStr">
+        <is>
+          <t>Thu  06/18</t>
+        </is>
+      </c>
+      <c r="C24" s="65" t="n"/>
+      <c r="D24" s="65" t="n"/>
+      <c r="E24" s="65" t="n"/>
+      <c r="F24" s="65" t="n"/>
+      <c r="G24" s="65" t="n"/>
+      <c r="H24" s="65" t="n"/>
+      <c r="I24" s="65" t="n"/>
+      <c r="J24" s="65" t="n"/>
+      <c r="K24" s="65" t="n"/>
+      <c r="L24" s="65" t="n"/>
+      <c r="M24" s="65" t="n"/>
+      <c r="N24" s="65" t="n"/>
+      <c r="O24" s="65" t="n"/>
+      <c r="P24" s="65" t="n"/>
+      <c r="Q24" s="65" t="n"/>
+      <c r="R24" s="65" t="n"/>
+      <c r="S24" s="65" t="n"/>
+      <c r="T24" s="65" t="n"/>
+      <c r="U24" s="65" t="n"/>
+      <c r="V24" s="65" t="n"/>
+      <c r="W24" s="65" t="n"/>
+      <c r="X24" s="65" t="n"/>
+      <c r="Y24" s="65" t="n"/>
+      <c r="Z24" s="65" t="n"/>
+      <c r="AA24" s="65" t="n"/>
+      <c r="AB24" s="65" t="n"/>
+    </row>
+    <row r="25" ht="16" customHeight="1">
+      <c r="B25" s="67" t="inlineStr">
+        <is>
+          <t>Fri  06/19</t>
+        </is>
+      </c>
+      <c r="C25" s="68" t="n"/>
+      <c r="D25" s="68" t="n"/>
+      <c r="E25" s="68" t="n"/>
+      <c r="F25" s="68" t="n"/>
+      <c r="G25" s="68" t="n"/>
+      <c r="H25" s="68" t="n"/>
+      <c r="I25" s="68" t="n"/>
+      <c r="J25" s="68" t="n"/>
+      <c r="K25" s="68" t="n"/>
+      <c r="L25" s="68" t="n"/>
+      <c r="M25" s="68" t="n"/>
+      <c r="N25" s="68" t="n"/>
+      <c r="O25" s="68" t="n"/>
+      <c r="P25" s="68" t="n"/>
+      <c r="Q25" s="68" t="n"/>
+      <c r="R25" s="68" t="n"/>
+      <c r="S25" s="68" t="n"/>
+      <c r="T25" s="68" t="n"/>
+      <c r="U25" s="68" t="n"/>
+      <c r="V25" s="68" t="n"/>
+      <c r="W25" s="68" t="n"/>
+      <c r="X25" s="68" t="n"/>
+      <c r="Y25" s="68" t="n"/>
+      <c r="Z25" s="68" t="n"/>
+      <c r="AA25" s="68" t="n"/>
+      <c r="AB25" s="68" t="n"/>
+    </row>
+    <row r="26" ht="4" customHeight="1"/>
+    <row r="27" ht="16" customHeight="1">
+      <c r="A27" s="53" t="inlineStr">
+        <is>
+          <t>Emma Wilson</t>
+        </is>
+      </c>
+      <c r="B27" s="54" t="inlineStr">
+        <is>
+          <t>Mon  06/15</t>
+        </is>
+      </c>
+      <c r="C27" s="57" t="n"/>
+      <c r="D27" s="57" t="n"/>
+      <c r="E27" s="57" t="n"/>
+      <c r="F27" s="57" t="n"/>
+      <c r="G27" s="55" t="n"/>
+      <c r="H27" s="55" t="n"/>
+      <c r="I27" s="55" t="n"/>
+      <c r="J27" s="55" t="n"/>
+      <c r="K27" s="55" t="n"/>
+      <c r="L27" s="55" t="n"/>
+      <c r="M27" s="55" t="n"/>
+      <c r="N27" s="55" t="n"/>
+      <c r="O27" s="56" t="n"/>
+      <c r="P27" s="55" t="n"/>
+      <c r="Q27" s="55" t="n"/>
+      <c r="R27" s="55" t="n"/>
+      <c r="S27" s="55" t="n"/>
+      <c r="T27" s="55" t="n"/>
+      <c r="U27" s="55" t="n"/>
+      <c r="V27" s="55" t="n"/>
+      <c r="W27" s="57" t="n"/>
+      <c r="X27" s="57" t="n"/>
+      <c r="Y27" s="57" t="n"/>
+      <c r="Z27" s="57" t="n"/>
+      <c r="AA27" s="57" t="n"/>
+      <c r="AB27" s="57" t="n"/>
+    </row>
+    <row r="28" ht="16" customHeight="1">
+      <c r="B28" s="58" t="inlineStr">
+        <is>
+          <t>Tue  06/16</t>
+        </is>
+      </c>
+      <c r="C28" s="57" t="n"/>
+      <c r="D28" s="57" t="n"/>
+      <c r="E28" s="57" t="n"/>
+      <c r="F28" s="57" t="n"/>
+      <c r="G28" s="55" t="n"/>
+      <c r="H28" s="55" t="n"/>
+      <c r="I28" s="55" t="n"/>
+      <c r="J28" s="55" t="n"/>
+      <c r="K28" s="55" t="n"/>
+      <c r="L28" s="55" t="n"/>
+      <c r="M28" s="55" t="n"/>
+      <c r="N28" s="55" t="n"/>
+      <c r="O28" s="56" t="n"/>
+      <c r="P28" s="55" t="n"/>
+      <c r="Q28" s="55" t="n"/>
+      <c r="R28" s="55" t="n"/>
+      <c r="S28" s="55" t="n"/>
+      <c r="T28" s="55" t="n"/>
+      <c r="U28" s="55" t="n"/>
+      <c r="V28" s="55" t="n"/>
+      <c r="W28" s="57" t="n"/>
+      <c r="X28" s="57" t="n"/>
+      <c r="Y28" s="57" t="n"/>
+      <c r="Z28" s="57" t="n"/>
+      <c r="AA28" s="57" t="n"/>
+      <c r="AB28" s="57" t="n"/>
+    </row>
+    <row r="29" ht="16" customHeight="1">
+      <c r="B29" s="58" t="inlineStr">
+        <is>
+          <t>Wed  06/17</t>
+        </is>
+      </c>
+      <c r="C29" s="57" t="n"/>
+      <c r="D29" s="57" t="n"/>
+      <c r="E29" s="57" t="n"/>
+      <c r="F29" s="57" t="n"/>
+      <c r="G29" s="55" t="n"/>
+      <c r="H29" s="55" t="n"/>
+      <c r="I29" s="55" t="n"/>
+      <c r="J29" s="55" t="n"/>
+      <c r="K29" s="55" t="n"/>
+      <c r="L29" s="55" t="n"/>
+      <c r="M29" s="55" t="n"/>
+      <c r="N29" s="55" t="n"/>
+      <c r="O29" s="56" t="n"/>
+      <c r="P29" s="55" t="n"/>
+      <c r="Q29" s="55" t="n"/>
+      <c r="R29" s="55" t="n"/>
+      <c r="S29" s="55" t="n"/>
+      <c r="T29" s="55" t="n"/>
+      <c r="U29" s="55" t="n"/>
+      <c r="V29" s="55" t="n"/>
+      <c r="W29" s="57" t="n"/>
+      <c r="X29" s="57" t="n"/>
+      <c r="Y29" s="57" t="n"/>
+      <c r="Z29" s="57" t="n"/>
+      <c r="AA29" s="57" t="n"/>
+      <c r="AB29" s="57" t="n"/>
+    </row>
+    <row r="30" ht="16" customHeight="1">
+      <c r="B30" s="58" t="inlineStr">
+        <is>
+          <t>Thu  06/18</t>
+        </is>
+      </c>
+      <c r="C30" s="57" t="n"/>
+      <c r="D30" s="57" t="n"/>
+      <c r="E30" s="57" t="n"/>
+      <c r="F30" s="57" t="n"/>
+      <c r="G30" s="57" t="n"/>
+      <c r="H30" s="57" t="n"/>
+      <c r="I30" s="57" t="n"/>
+      <c r="J30" s="57" t="n"/>
+      <c r="K30" s="57" t="n"/>
+      <c r="L30" s="57" t="n"/>
+      <c r="M30" s="57" t="n"/>
+      <c r="N30" s="57" t="n"/>
+      <c r="O30" s="57" t="n"/>
+      <c r="P30" s="57" t="n"/>
+      <c r="Q30" s="57" t="n"/>
+      <c r="R30" s="57" t="n"/>
+      <c r="S30" s="57" t="n"/>
+      <c r="T30" s="57" t="n"/>
+      <c r="U30" s="57" t="n"/>
+      <c r="V30" s="57" t="n"/>
+      <c r="W30" s="57" t="n"/>
+      <c r="X30" s="57" t="n"/>
+      <c r="Y30" s="57" t="n"/>
+      <c r="Z30" s="57" t="n"/>
+      <c r="AA30" s="57" t="n"/>
+      <c r="AB30" s="57" t="n"/>
+    </row>
+    <row r="31" ht="16" customHeight="1">
+      <c r="B31" s="59" t="inlineStr">
+        <is>
+          <t>Fri  06/19</t>
+        </is>
+      </c>
+      <c r="C31" s="62" t="n"/>
+      <c r="D31" s="62" t="n"/>
+      <c r="E31" s="62" t="n"/>
+      <c r="F31" s="62" t="n"/>
+      <c r="G31" s="60" t="n"/>
+      <c r="H31" s="60" t="n"/>
+      <c r="I31" s="60" t="n"/>
+      <c r="J31" s="60" t="n"/>
+      <c r="K31" s="60" t="n"/>
+      <c r="L31" s="60" t="n"/>
+      <c r="M31" s="60" t="n"/>
+      <c r="N31" s="60" t="n"/>
+      <c r="O31" s="61" t="n"/>
+      <c r="P31" s="60" t="n"/>
+      <c r="Q31" s="60" t="n"/>
+      <c r="R31" s="60" t="n"/>
+      <c r="S31" s="60" t="n"/>
+      <c r="T31" s="60" t="n"/>
+      <c r="U31" s="60" t="n"/>
+      <c r="V31" s="60" t="n"/>
+      <c r="W31" s="62" t="n"/>
+      <c r="X31" s="62" t="n"/>
+      <c r="Y31" s="62" t="n"/>
+      <c r="Z31" s="62" t="n"/>
+      <c r="AA31" s="62" t="n"/>
+      <c r="AB31" s="62" t="n"/>
+    </row>
+    <row r="32" ht="4" customHeight="1"/>
+    <row r="33" ht="16" customHeight="1">
+      <c r="A33" s="63" t="inlineStr">
+        <is>
+          <t>Frank Brown</t>
+        </is>
+      </c>
+      <c r="B33" s="64" t="inlineStr">
+        <is>
+          <t>Mon  06/15</t>
+        </is>
+      </c>
+      <c r="C33" s="55" t="n"/>
+      <c r="D33" s="55" t="n"/>
+      <c r="E33" s="55" t="n"/>
+      <c r="F33" s="55" t="n"/>
+      <c r="G33" s="55" t="n"/>
+      <c r="H33" s="55" t="n"/>
+      <c r="I33" s="55" t="n"/>
+      <c r="J33" s="55" t="n"/>
+      <c r="K33" s="56" t="n"/>
+      <c r="L33" s="55" t="n"/>
+      <c r="M33" s="55" t="n"/>
+      <c r="N33" s="55" t="n"/>
+      <c r="O33" s="55" t="n"/>
+      <c r="P33" s="55" t="n"/>
+      <c r="Q33" s="55" t="n"/>
+      <c r="R33" s="55" t="n"/>
+      <c r="S33" s="65" t="n"/>
+      <c r="T33" s="65" t="n"/>
+      <c r="U33" s="65" t="n"/>
+      <c r="V33" s="65" t="n"/>
+      <c r="W33" s="65" t="n"/>
+      <c r="X33" s="65" t="n"/>
+      <c r="Y33" s="65" t="n"/>
+      <c r="Z33" s="65" t="n"/>
+      <c r="AA33" s="65" t="n"/>
+      <c r="AB33" s="65" t="n"/>
+    </row>
+    <row r="34" ht="16" customHeight="1">
+      <c r="B34" s="66" t="inlineStr">
+        <is>
+          <t>Tue  06/16</t>
+        </is>
+      </c>
+      <c r="C34" s="55" t="n"/>
+      <c r="D34" s="55" t="n"/>
+      <c r="E34" s="55" t="n"/>
+      <c r="F34" s="55" t="n"/>
+      <c r="G34" s="55" t="n"/>
+      <c r="H34" s="55" t="n"/>
+      <c r="I34" s="55" t="n"/>
+      <c r="J34" s="55" t="n"/>
+      <c r="K34" s="56" t="n"/>
+      <c r="L34" s="55" t="n"/>
+      <c r="M34" s="55" t="n"/>
+      <c r="N34" s="55" t="n"/>
+      <c r="O34" s="55" t="n"/>
+      <c r="P34" s="55" t="n"/>
+      <c r="Q34" s="55" t="n"/>
+      <c r="R34" s="55" t="n"/>
+      <c r="S34" s="65" t="n"/>
+      <c r="T34" s="65" t="n"/>
+      <c r="U34" s="65" t="n"/>
+      <c r="V34" s="65" t="n"/>
+      <c r="W34" s="65" t="n"/>
+      <c r="X34" s="65" t="n"/>
+      <c r="Y34" s="65" t="n"/>
+      <c r="Z34" s="65" t="n"/>
+      <c r="AA34" s="65" t="n"/>
+      <c r="AB34" s="65" t="n"/>
+    </row>
+    <row r="35" ht="16" customHeight="1">
+      <c r="B35" s="66" t="inlineStr">
+        <is>
+          <t>Wed  06/17</t>
+        </is>
+      </c>
+      <c r="C35" s="65" t="n"/>
+      <c r="D35" s="65" t="n"/>
+      <c r="E35" s="65" t="n"/>
+      <c r="F35" s="65" t="n"/>
+      <c r="G35" s="65" t="n"/>
+      <c r="H35" s="65" t="n"/>
+      <c r="I35" s="65" t="n"/>
+      <c r="J35" s="65" t="n"/>
+      <c r="K35" s="65" t="n"/>
+      <c r="L35" s="65" t="n"/>
+      <c r="M35" s="65" t="n"/>
+      <c r="N35" s="65" t="n"/>
+      <c r="O35" s="65" t="n"/>
+      <c r="P35" s="65" t="n"/>
+      <c r="Q35" s="65" t="n"/>
+      <c r="R35" s="65" t="n"/>
+      <c r="S35" s="65" t="n"/>
+      <c r="T35" s="65" t="n"/>
+      <c r="U35" s="65" t="n"/>
+      <c r="V35" s="65" t="n"/>
+      <c r="W35" s="65" t="n"/>
+      <c r="X35" s="65" t="n"/>
+      <c r="Y35" s="65" t="n"/>
+      <c r="Z35" s="65" t="n"/>
+      <c r="AA35" s="65" t="n"/>
+      <c r="AB35" s="65" t="n"/>
+    </row>
+    <row r="36" ht="16" customHeight="1">
+      <c r="B36" s="66" t="inlineStr">
+        <is>
+          <t>Thu  06/18</t>
+        </is>
+      </c>
+      <c r="C36" s="55" t="n"/>
+      <c r="D36" s="55" t="n"/>
+      <c r="E36" s="55" t="n"/>
+      <c r="F36" s="55" t="n"/>
+      <c r="G36" s="55" t="n"/>
+      <c r="H36" s="55" t="n"/>
+      <c r="I36" s="55" t="n"/>
+      <c r="J36" s="55" t="n"/>
+      <c r="K36" s="56" t="n"/>
+      <c r="L36" s="55" t="n"/>
+      <c r="M36" s="55" t="n"/>
+      <c r="N36" s="55" t="n"/>
+      <c r="O36" s="55" t="n"/>
+      <c r="P36" s="55" t="n"/>
+      <c r="Q36" s="55" t="n"/>
+      <c r="R36" s="55" t="n"/>
+      <c r="S36" s="65" t="n"/>
+      <c r="T36" s="65" t="n"/>
+      <c r="U36" s="65" t="n"/>
+      <c r="V36" s="65" t="n"/>
+      <c r="W36" s="65" t="n"/>
+      <c r="X36" s="65" t="n"/>
+      <c r="Y36" s="65" t="n"/>
+      <c r="Z36" s="65" t="n"/>
+      <c r="AA36" s="65" t="n"/>
+      <c r="AB36" s="65" t="n"/>
+    </row>
+    <row r="37" ht="16" customHeight="1">
+      <c r="B37" s="67" t="inlineStr">
+        <is>
+          <t>Fri  06/19</t>
+        </is>
+      </c>
+      <c r="C37" s="60" t="n"/>
+      <c r="D37" s="60" t="n"/>
+      <c r="E37" s="60" t="n"/>
+      <c r="F37" s="60" t="n"/>
+      <c r="G37" s="60" t="n"/>
+      <c r="H37" s="60" t="n"/>
+      <c r="I37" s="60" t="n"/>
+      <c r="J37" s="60" t="n"/>
+      <c r="K37" s="61" t="n"/>
+      <c r="L37" s="60" t="n"/>
+      <c r="M37" s="60" t="n"/>
+      <c r="N37" s="60" t="n"/>
+      <c r="O37" s="60" t="n"/>
+      <c r="P37" s="60" t="n"/>
+      <c r="Q37" s="60" t="n"/>
+      <c r="R37" s="60" t="n"/>
+      <c r="S37" s="68" t="n"/>
+      <c r="T37" s="68" t="n"/>
+      <c r="U37" s="68" t="n"/>
+      <c r="V37" s="68" t="n"/>
+      <c r="W37" s="68" t="n"/>
+      <c r="X37" s="68" t="n"/>
+      <c r="Y37" s="68" t="n"/>
+      <c r="Z37" s="68" t="n"/>
+      <c r="AA37" s="68" t="n"/>
+      <c r="AB37" s="68" t="n"/>
+    </row>
+    <row r="38" ht="4" customHeight="1"/>
+    <row r="39" ht="16" customHeight="1">
+      <c r="A39" s="53" t="inlineStr">
+        <is>
+          <t>Grace Kim</t>
+        </is>
+      </c>
+      <c r="B39" s="54" t="inlineStr">
+        <is>
+          <t>Mon  06/15</t>
+        </is>
+      </c>
+      <c r="C39" s="55" t="n"/>
+      <c r="D39" s="55" t="n"/>
+      <c r="E39" s="55" t="n"/>
+      <c r="F39" s="55" t="n"/>
+      <c r="G39" s="55" t="n"/>
+      <c r="H39" s="55" t="n"/>
+      <c r="I39" s="56" t="n"/>
+      <c r="J39" s="55" t="n"/>
+      <c r="K39" s="55" t="n"/>
+      <c r="L39" s="55" t="n"/>
+      <c r="M39" s="55" t="n"/>
+      <c r="N39" s="55" t="n"/>
+      <c r="O39" s="57" t="n"/>
+      <c r="P39" s="57" t="n"/>
+      <c r="Q39" s="57" t="n"/>
+      <c r="R39" s="57" t="n"/>
+      <c r="S39" s="57" t="n"/>
+      <c r="T39" s="57" t="n"/>
+      <c r="U39" s="57" t="n"/>
+      <c r="V39" s="57" t="n"/>
+      <c r="W39" s="57" t="n"/>
+      <c r="X39" s="57" t="n"/>
+      <c r="Y39" s="57" t="n"/>
+      <c r="Z39" s="57" t="n"/>
+      <c r="AA39" s="57" t="n"/>
+      <c r="AB39" s="57" t="n"/>
+    </row>
+    <row r="40" ht="16" customHeight="1">
+      <c r="B40" s="58" t="inlineStr">
+        <is>
+          <t>Tue  06/16</t>
+        </is>
+      </c>
+      <c r="C40" s="57" t="n"/>
+      <c r="D40" s="57" t="n"/>
+      <c r="E40" s="57" t="n"/>
+      <c r="F40" s="57" t="n"/>
+      <c r="G40" s="57" t="n"/>
+      <c r="H40" s="57" t="n"/>
+      <c r="I40" s="57" t="n"/>
+      <c r="J40" s="57" t="n"/>
+      <c r="K40" s="57" t="n"/>
+      <c r="L40" s="57" t="n"/>
+      <c r="M40" s="57" t="n"/>
+      <c r="N40" s="57" t="n"/>
+      <c r="O40" s="57" t="n"/>
+      <c r="P40" s="57" t="n"/>
+      <c r="Q40" s="57" t="n"/>
+      <c r="R40" s="57" t="n"/>
+      <c r="S40" s="57" t="n"/>
+      <c r="T40" s="57" t="n"/>
+      <c r="U40" s="57" t="n"/>
+      <c r="V40" s="57" t="n"/>
+      <c r="W40" s="57" t="n"/>
+      <c r="X40" s="57" t="n"/>
+      <c r="Y40" s="57" t="n"/>
+      <c r="Z40" s="57" t="n"/>
+      <c r="AA40" s="57" t="n"/>
+      <c r="AB40" s="57" t="n"/>
+    </row>
+    <row r="41" ht="16" customHeight="1">
+      <c r="B41" s="58" t="inlineStr">
+        <is>
+          <t>Wed  06/17</t>
+        </is>
+      </c>
+      <c r="C41" s="55" t="n"/>
+      <c r="D41" s="55" t="n"/>
+      <c r="E41" s="55" t="n"/>
+      <c r="F41" s="55" t="n"/>
+      <c r="G41" s="55" t="n"/>
+      <c r="H41" s="55" t="n"/>
+      <c r="I41" s="56" t="n"/>
+      <c r="J41" s="55" t="n"/>
+      <c r="K41" s="55" t="n"/>
+      <c r="L41" s="55" t="n"/>
+      <c r="M41" s="55" t="n"/>
+      <c r="N41" s="55" t="n"/>
+      <c r="O41" s="57" t="n"/>
+      <c r="P41" s="57" t="n"/>
+      <c r="Q41" s="57" t="n"/>
+      <c r="R41" s="57" t="n"/>
+      <c r="S41" s="57" t="n"/>
+      <c r="T41" s="57" t="n"/>
+      <c r="U41" s="57" t="n"/>
+      <c r="V41" s="57" t="n"/>
+      <c r="W41" s="57" t="n"/>
+      <c r="X41" s="57" t="n"/>
+      <c r="Y41" s="57" t="n"/>
+      <c r="Z41" s="57" t="n"/>
+      <c r="AA41" s="57" t="n"/>
+      <c r="AB41" s="57" t="n"/>
+    </row>
+    <row r="42" ht="16" customHeight="1">
+      <c r="B42" s="58" t="inlineStr">
+        <is>
+          <t>Thu  06/18</t>
+        </is>
+      </c>
+      <c r="C42" s="55" t="n"/>
+      <c r="D42" s="55" t="n"/>
+      <c r="E42" s="55" t="n"/>
+      <c r="F42" s="55" t="n"/>
+      <c r="G42" s="55" t="n"/>
+      <c r="H42" s="55" t="n"/>
+      <c r="I42" s="56" t="n"/>
+      <c r="J42" s="55" t="n"/>
+      <c r="K42" s="55" t="n"/>
+      <c r="L42" s="55" t="n"/>
+      <c r="M42" s="55" t="n"/>
+      <c r="N42" s="55" t="n"/>
+      <c r="O42" s="57" t="n"/>
+      <c r="P42" s="57" t="n"/>
+      <c r="Q42" s="57" t="n"/>
+      <c r="R42" s="57" t="n"/>
+      <c r="S42" s="57" t="n"/>
+      <c r="T42" s="57" t="n"/>
+      <c r="U42" s="57" t="n"/>
+      <c r="V42" s="57" t="n"/>
+      <c r="W42" s="57" t="n"/>
+      <c r="X42" s="57" t="n"/>
+      <c r="Y42" s="57" t="n"/>
+      <c r="Z42" s="57" t="n"/>
+      <c r="AA42" s="57" t="n"/>
+      <c r="AB42" s="57" t="n"/>
+    </row>
+    <row r="43" ht="16" customHeight="1">
+      <c r="B43" s="59" t="inlineStr">
+        <is>
+          <t>Fri  06/19</t>
+        </is>
+      </c>
+      <c r="C43" s="62" t="n"/>
+      <c r="D43" s="62" t="n"/>
+      <c r="E43" s="62" t="n"/>
+      <c r="F43" s="62" t="n"/>
+      <c r="G43" s="62" t="n"/>
+      <c r="H43" s="62" t="n"/>
+      <c r="I43" s="62" t="n"/>
+      <c r="J43" s="62" t="n"/>
+      <c r="K43" s="62" t="n"/>
+      <c r="L43" s="62" t="n"/>
+      <c r="M43" s="62" t="n"/>
+      <c r="N43" s="62" t="n"/>
+      <c r="O43" s="62" t="n"/>
+      <c r="P43" s="62" t="n"/>
+      <c r="Q43" s="62" t="n"/>
+      <c r="R43" s="62" t="n"/>
+      <c r="S43" s="62" t="n"/>
+      <c r="T43" s="62" t="n"/>
+      <c r="U43" s="62" t="n"/>
+      <c r="V43" s="62" t="n"/>
+      <c r="W43" s="62" t="n"/>
+      <c r="X43" s="62" t="n"/>
+      <c r="Y43" s="62" t="n"/>
+      <c r="Z43" s="62" t="n"/>
+      <c r="AA43" s="62" t="n"/>
+      <c r="AB43" s="62" t="n"/>
+    </row>
+    <row r="44" ht="4" customHeight="1"/>
+    <row r="45" ht="16" customHeight="1">
+      <c r="A45" s="63" t="inlineStr">
+        <is>
+          <t>Henry Davis</t>
+        </is>
+      </c>
+      <c r="B45" s="64" t="inlineStr">
+        <is>
+          <t>Mon  06/15</t>
+        </is>
+      </c>
+      <c r="C45" s="65" t="n"/>
+      <c r="D45" s="65" t="n"/>
+      <c r="E45" s="65" t="n"/>
+      <c r="F45" s="65" t="n"/>
+      <c r="G45" s="65" t="n"/>
+      <c r="H45" s="65" t="n"/>
+      <c r="I45" s="65" t="n"/>
+      <c r="J45" s="65" t="n"/>
+      <c r="K45" s="65" t="n"/>
+      <c r="L45" s="65" t="n"/>
+      <c r="M45" s="65" t="n"/>
+      <c r="N45" s="65" t="n"/>
+      <c r="O45" s="55" t="n"/>
+      <c r="P45" s="55" t="n"/>
+      <c r="Q45" s="55" t="n"/>
+      <c r="R45" s="55" t="n"/>
+      <c r="S45" s="55" t="n"/>
+      <c r="T45" s="55" t="n"/>
+      <c r="U45" s="55" t="n"/>
+      <c r="V45" s="56" t="n"/>
+      <c r="W45" s="55" t="n"/>
+      <c r="X45" s="55" t="n"/>
+      <c r="Y45" s="55" t="n"/>
+      <c r="Z45" s="55" t="n"/>
+      <c r="AA45" s="55" t="n"/>
+      <c r="AB45" s="55" t="n"/>
+    </row>
+    <row r="46" ht="16" customHeight="1">
+      <c r="B46" s="66" t="inlineStr">
+        <is>
+          <t>Tue  06/16</t>
+        </is>
+      </c>
+      <c r="C46" s="65" t="n"/>
+      <c r="D46" s="65" t="n"/>
+      <c r="E46" s="65" t="n"/>
+      <c r="F46" s="65" t="n"/>
+      <c r="G46" s="65" t="n"/>
+      <c r="H46" s="65" t="n"/>
+      <c r="I46" s="65" t="n"/>
+      <c r="J46" s="65" t="n"/>
+      <c r="K46" s="65" t="n"/>
+      <c r="L46" s="65" t="n"/>
+      <c r="M46" s="65" t="n"/>
+      <c r="N46" s="65" t="n"/>
+      <c r="O46" s="55" t="n"/>
+      <c r="P46" s="55" t="n"/>
+      <c r="Q46" s="55" t="n"/>
+      <c r="R46" s="55" t="n"/>
+      <c r="S46" s="55" t="n"/>
+      <c r="T46" s="55" t="n"/>
+      <c r="U46" s="55" t="n"/>
+      <c r="V46" s="56" t="n"/>
+      <c r="W46" s="55" t="n"/>
+      <c r="X46" s="55" t="n"/>
+      <c r="Y46" s="55" t="n"/>
+      <c r="Z46" s="55" t="n"/>
+      <c r="AA46" s="55" t="n"/>
+      <c r="AB46" s="55" t="n"/>
+    </row>
+    <row r="47" ht="16" customHeight="1">
+      <c r="B47" s="66" t="inlineStr">
+        <is>
+          <t>Wed  06/17</t>
+        </is>
+      </c>
+      <c r="C47" s="65" t="n"/>
+      <c r="D47" s="65" t="n"/>
+      <c r="E47" s="65" t="n"/>
+      <c r="F47" s="65" t="n"/>
+      <c r="G47" s="65" t="n"/>
+      <c r="H47" s="65" t="n"/>
+      <c r="I47" s="65" t="n"/>
+      <c r="J47" s="65" t="n"/>
+      <c r="K47" s="65" t="n"/>
+      <c r="L47" s="65" t="n"/>
+      <c r="M47" s="65" t="n"/>
+      <c r="N47" s="65" t="n"/>
+      <c r="O47" s="55" t="n"/>
+      <c r="P47" s="55" t="n"/>
+      <c r="Q47" s="55" t="n"/>
+      <c r="R47" s="55" t="n"/>
+      <c r="S47" s="55" t="n"/>
+      <c r="T47" s="55" t="n"/>
+      <c r="U47" s="55" t="n"/>
+      <c r="V47" s="56" t="n"/>
+      <c r="W47" s="55" t="n"/>
+      <c r="X47" s="55" t="n"/>
+      <c r="Y47" s="55" t="n"/>
+      <c r="Z47" s="55" t="n"/>
+      <c r="AA47" s="55" t="n"/>
+      <c r="AB47" s="55" t="n"/>
+    </row>
+    <row r="48" ht="16" customHeight="1">
+      <c r="B48" s="66" t="inlineStr">
+        <is>
+          <t>Thu  06/18</t>
+        </is>
+      </c>
+      <c r="C48" s="65" t="n"/>
+      <c r="D48" s="65" t="n"/>
+      <c r="E48" s="65" t="n"/>
+      <c r="F48" s="65" t="n"/>
+      <c r="G48" s="65" t="n"/>
+      <c r="H48" s="65" t="n"/>
+      <c r="I48" s="65" t="n"/>
+      <c r="J48" s="65" t="n"/>
+      <c r="K48" s="65" t="n"/>
+      <c r="L48" s="65" t="n"/>
+      <c r="M48" s="65" t="n"/>
+      <c r="N48" s="65" t="n"/>
+      <c r="O48" s="65" t="n"/>
+      <c r="P48" s="65" t="n"/>
+      <c r="Q48" s="65" t="n"/>
+      <c r="R48" s="65" t="n"/>
+      <c r="S48" s="65" t="n"/>
+      <c r="T48" s="65" t="n"/>
+      <c r="U48" s="65" t="n"/>
+      <c r="V48" s="65" t="n"/>
+      <c r="W48" s="65" t="n"/>
+      <c r="X48" s="65" t="n"/>
+      <c r="Y48" s="65" t="n"/>
+      <c r="Z48" s="65" t="n"/>
+      <c r="AA48" s="65" t="n"/>
+      <c r="AB48" s="65" t="n"/>
+    </row>
+    <row r="49" ht="16" customHeight="1">
+      <c r="B49" s="67" t="inlineStr">
+        <is>
+          <t>Fri  06/19</t>
+        </is>
+      </c>
+      <c r="C49" s="68" t="n"/>
+      <c r="D49" s="68" t="n"/>
+      <c r="E49" s="68" t="n"/>
+      <c r="F49" s="68" t="n"/>
+      <c r="G49" s="68" t="n"/>
+      <c r="H49" s="68" t="n"/>
+      <c r="I49" s="68" t="n"/>
+      <c r="J49" s="68" t="n"/>
+      <c r="K49" s="68" t="n"/>
+      <c r="L49" s="68" t="n"/>
+      <c r="M49" s="68" t="n"/>
+      <c r="N49" s="68" t="n"/>
+      <c r="O49" s="60" t="n"/>
+      <c r="P49" s="60" t="n"/>
+      <c r="Q49" s="60" t="n"/>
+      <c r="R49" s="60" t="n"/>
+      <c r="S49" s="60" t="n"/>
+      <c r="T49" s="60" t="n"/>
+      <c r="U49" s="60" t="n"/>
+      <c r="V49" s="61" t="n"/>
+      <c r="W49" s="60" t="n"/>
+      <c r="X49" s="60" t="n"/>
+      <c r="Y49" s="60" t="n"/>
+      <c r="Z49" s="60" t="n"/>
+      <c r="AA49" s="60" t="n"/>
+      <c r="AB49" s="60" t="n"/>
+    </row>
+    <row r="50" ht="4" customHeight="1"/>
+    <row r="52" ht="16" customHeight="1">
+      <c r="A52" s="69" t="inlineStr">
+        <is>
+          <t>Legend:</t>
+        </is>
+      </c>
+      <c r="C52" s="70" t="n"/>
+      <c r="D52" s="71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  On Shift</t>
+        </is>
+      </c>
+      <c r="F52" s="72" t="n"/>
+      <c r="G52" s="71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Lunch (estimated midpoint)</t>
+        </is>
+      </c>
+      <c r="I52" s="73" t="n"/>
+      <c r="J52" s="71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Off / Not Working</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A21:A25"/>
+    <mergeCell ref="A39:A43"/>
+    <mergeCell ref="A15:A19"/>
+    <mergeCell ref="A9:A13"/>
+    <mergeCell ref="A27:A31"/>
+    <mergeCell ref="A1:AB1"/>
+    <mergeCell ref="A3:A7"/>
+    <mergeCell ref="A33:A37"/>
+    <mergeCell ref="A45:A49"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>